<commit_message>
DC Jack Link added in Client BOM
</commit_message>
<xml_diff>
--- a/Design Files/BLE_product-v1.0/Deliverables/BOM/Client BOM.xlsx
+++ b/Design Files/BLE_product-v1.0/Deliverables/BOM/Client BOM.xlsx
@@ -1,25 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26924"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\raafat-BLEproduct\Design Files\BLE_product-v1.0\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\eSpark-Consultants\raafat-BLEproduct\Design Files\BLE_product-v1.0\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3202CC14-5577-4070-8CA0-241BAFC8B6E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="156">
   <si>
     <t>#</t>
   </si>
@@ -492,7 +504,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -758,7 +770,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -839,24 +851,25 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1143,9 +1156,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:P35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="7" customWidth="1"/>
@@ -1161,7 +1174,7 @@
     <col min="12" max="12" width="8.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -1170,12 +1183,12 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
-      <c r="K1" s="27"/>
-      <c r="L1" s="27"/>
-    </row>
-    <row r="2" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
+      <c r="K1" s="32"/>
+      <c r="L1" s="32"/>
+    </row>
+    <row r="2" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="8" t="s">
         <v>0</v>
@@ -1211,7 +1224,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="23">
         <f>ROW(B3) - ROW($B$2)</f>
@@ -1244,7 +1257,7 @@
       <c r="K3" s="15"/>
       <c r="L3" s="15"/>
     </row>
-    <row r="4" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="23">
         <f t="shared" ref="B4:B30" si="0">ROW(B4) - ROW($B$2)</f>
@@ -1277,7 +1290,7 @@
       <c r="K4" s="17"/>
       <c r="L4" s="17"/>
     </row>
-    <row r="5" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="B5" s="23">
         <f>ROW(B5) - ROW($B$2)</f>
@@ -1310,7 +1323,7 @@
       <c r="K5" s="15"/>
       <c r="L5" s="15"/>
     </row>
-    <row r="6" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="B6" s="23">
         <f t="shared" si="0"/>
@@ -1343,7 +1356,7 @@
       <c r="K6" s="17"/>
       <c r="L6" s="17"/>
     </row>
-    <row r="7" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="B7" s="23">
         <f>ROW(B7) - ROW($B$2)</f>
@@ -1376,7 +1389,7 @@
       <c r="K7" s="15"/>
       <c r="L7" s="15"/>
     </row>
-    <row r="8" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="23">
         <f t="shared" si="0"/>
@@ -1409,7 +1422,7 @@
       <c r="K8" s="17"/>
       <c r="L8" s="17"/>
     </row>
-    <row r="9" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="23">
         <f>ROW(B9) - ROW($B$2)</f>
@@ -1442,7 +1455,7 @@
       <c r="K9" s="15"/>
       <c r="L9" s="15"/>
     </row>
-    <row r="10" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="23">
         <f t="shared" si="0"/>
@@ -1451,31 +1464,31 @@
       <c r="C10" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="D10" s="28" t="s">
+      <c r="D10" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="E10" s="29" t="s">
+      <c r="E10" s="28" t="s">
         <v>50</v>
       </c>
-      <c r="F10" s="28" t="s">
+      <c r="F10" s="27" t="s">
         <v>76</v>
       </c>
-      <c r="G10" s="29" t="s">
+      <c r="G10" s="28" t="s">
         <v>76</v>
       </c>
-      <c r="H10" s="28" t="s">
+      <c r="H10" s="27" t="s">
         <v>150</v>
       </c>
-      <c r="I10" s="29"/>
-      <c r="J10" s="28">
+      <c r="I10" s="28"/>
+      <c r="J10" s="27">
         <v>4</v>
       </c>
       <c r="K10" s="17"/>
-      <c r="L10" s="30" t="s">
+      <c r="L10" s="29" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="23">
         <f>ROW(B11) - ROW($B$2)</f>
@@ -1503,10 +1516,12 @@
       <c r="J11" s="15">
         <v>1</v>
       </c>
-      <c r="K11" s="15"/>
+      <c r="K11" s="26" t="s">
+        <v>152</v>
+      </c>
       <c r="L11" s="15"/>
     </row>
-    <row r="12" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="23">
         <f t="shared" si="0"/>
@@ -1515,54 +1530,55 @@
       <c r="C12" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="D12" s="28" t="s">
+      <c r="D12" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="E12" s="29" t="s">
+      <c r="E12" s="28" t="s">
         <v>52</v>
       </c>
-      <c r="F12" s="28" t="s">
+      <c r="F12" s="27" t="s">
         <v>78</v>
       </c>
-      <c r="G12" s="29" t="s">
+      <c r="G12" s="28" t="s">
         <v>101</v>
       </c>
-      <c r="H12" s="28"/>
-      <c r="I12" s="29"/>
-      <c r="J12" s="28">
-        <v>1</v>
-      </c>
-      <c r="K12" s="28"/>
-      <c r="L12" s="30" t="s">
+      <c r="H12" s="27"/>
+      <c r="I12" s="28"/>
+      <c r="J12" s="27">
+        <v>1</v>
+      </c>
+      <c r="K12" s="27"/>
+      <c r="L12" s="29" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="23">
         <f>ROW(B13) - ROW($B$2)</f>
         <v>11</v>
       </c>
       <c r="C13" s="25"/>
-      <c r="D13" s="31" t="s">
+      <c r="D13" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="E13" s="32"/>
-      <c r="F13" s="31" t="s">
+      <c r="E13" s="31"/>
+      <c r="F13" s="30" t="s">
         <v>79</v>
       </c>
-      <c r="G13" s="32"/>
-      <c r="H13" s="31"/>
-      <c r="I13" s="32"/>
-      <c r="J13" s="31">
-        <v>1</v>
-      </c>
-      <c r="K13" s="31"/>
-      <c r="L13" s="30" t="s">
+      <c r="G13" s="31"/>
+      <c r="H13" s="30"/>
+      <c r="I13" s="31"/>
+      <c r="J13" s="30">
+        <v>1</v>
+      </c>
+      <c r="K13" s="30"/>
+      <c r="L13" s="29" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="14" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P13" s="33"/>
+    </row>
+    <row r="14" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="23">
         <f t="shared" si="0"/>
@@ -1593,7 +1609,7 @@
       <c r="K14" s="17"/>
       <c r="L14" s="17"/>
     </row>
-    <row r="15" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:16" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="23">
         <f>ROW(B15) - ROW($B$2)</f>
@@ -1624,7 +1640,7 @@
       <c r="K15" s="15"/>
       <c r="L15" s="15"/>
     </row>
-    <row r="16" spans="1:12" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="23">
         <f t="shared" si="0"/>
@@ -2223,10 +2239,11 @@
     <mergeCell ref="I1:L1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="K32" r:id="rId1"/>
-    <hyperlink ref="K33" r:id="rId2"/>
+    <hyperlink ref="K32" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="K33" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="K11" r:id="rId3" xr:uid="{7163F1D9-70FF-4B1B-8161-0B8D0362F853}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
#6 U4 Updated BOM and Schematic.
</commit_message>
<xml_diff>
--- a/Design Files/BLE_product-v1.0/Deliverables/BOM/Client BOM.xlsx
+++ b/Design Files/BLE_product-v1.0/Deliverables/BOM/Client BOM.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26924"/>
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\eSpark-Consultants\raafat-BLEproduct\Design Files\BLE_product-v1.0\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\raafat-BLEproduct\Design Files\BLE_product-v1.0\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3202CC14-5577-4070-8CA0-241BAFC8B6E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -31,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="156">
   <si>
     <t>#</t>
   </si>
@@ -372,9 +371,6 @@
     <t>TLV73330PDQNR</t>
   </si>
   <si>
-    <t>FAN54120UC420X</t>
-  </si>
-  <si>
     <t>CSD25501F3</t>
   </si>
   <si>
@@ -499,12 +495,15 @@
   </si>
   <si>
     <t>DNP</t>
+  </si>
+  <si>
+    <t>FAN54120MP420X</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -770,7 +769,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -869,7 +868,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1156,9 +1154,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:P35"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="7" customWidth="1"/>
@@ -1172,9 +1170,10 @@
     <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="25.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -1188,7 +1187,7 @@
       <c r="K1" s="32"/>
       <c r="L1" s="32"/>
     </row>
-    <row r="2" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="8" t="s">
         <v>0</v>
@@ -1209,22 +1208,22 @@
         <v>94</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I2" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="L2" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="J2" s="8" t="s">
-        <v>145</v>
-      </c>
-      <c r="K2" s="8" t="s">
-        <v>151</v>
-      </c>
-      <c r="L2" s="8" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="23">
         <f>ROW(B3) - ROW($B$2)</f>
@@ -1246,10 +1245,10 @@
         <v>95</v>
       </c>
       <c r="H3" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I3" s="16" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="J3" s="15">
         <v>6</v>
@@ -1257,7 +1256,7 @@
       <c r="K3" s="15"/>
       <c r="L3" s="15"/>
     </row>
-    <row r="4" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="23">
         <f t="shared" ref="B4:B30" si="0">ROW(B4) - ROW($B$2)</f>
@@ -1279,10 +1278,10 @@
         <v>96</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="I4" s="18" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="J4" s="17">
         <v>1</v>
@@ -1290,7 +1289,7 @@
       <c r="K4" s="17"/>
       <c r="L4" s="17"/>
     </row>
-    <row r="5" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="B5" s="23">
         <f>ROW(B5) - ROW($B$2)</f>
@@ -1312,10 +1311,10 @@
         <v>97</v>
       </c>
       <c r="H5" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I5" s="16" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="J5" s="15">
         <v>1</v>
@@ -1323,7 +1322,7 @@
       <c r="K5" s="15"/>
       <c r="L5" s="15"/>
     </row>
-    <row r="6" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="B6" s="23">
         <f t="shared" si="0"/>
@@ -1345,10 +1344,10 @@
         <v>98</v>
       </c>
       <c r="H6" s="17" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I6" s="18" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="J6" s="17">
         <v>1</v>
@@ -1356,7 +1355,7 @@
       <c r="K6" s="17"/>
       <c r="L6" s="17"/>
     </row>
-    <row r="7" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="B7" s="23">
         <f>ROW(B7) - ROW($B$2)</f>
@@ -1378,10 +1377,10 @@
         <v>99</v>
       </c>
       <c r="H7" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I7" s="16" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="J7" s="15">
         <v>1</v>
@@ -1389,7 +1388,7 @@
       <c r="K7" s="15"/>
       <c r="L7" s="15"/>
     </row>
-    <row r="8" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="23">
         <f t="shared" si="0"/>
@@ -1411,10 +1410,10 @@
         <v>75</v>
       </c>
       <c r="H8" s="17" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I8" s="18" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="J8" s="17">
         <v>1</v>
@@ -1422,7 +1421,7 @@
       <c r="K8" s="17"/>
       <c r="L8" s="17"/>
     </row>
-    <row r="9" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="23">
         <f>ROW(B9) - ROW($B$2)</f>
@@ -1444,10 +1443,10 @@
         <v>100</v>
       </c>
       <c r="H9" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I9" s="16" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="J9" s="15">
         <v>1</v>
@@ -1455,7 +1454,7 @@
       <c r="K9" s="15"/>
       <c r="L9" s="15"/>
     </row>
-    <row r="10" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="23">
         <f t="shared" si="0"/>
@@ -1477,7 +1476,7 @@
         <v>76</v>
       </c>
       <c r="H10" s="27" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="I10" s="28"/>
       <c r="J10" s="27">
@@ -1485,10 +1484,10 @@
       </c>
       <c r="K10" s="17"/>
       <c r="L10" s="29" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="23">
         <f>ROW(B11) - ROW($B$2)</f>
@@ -1510,18 +1509,18 @@
         <v>77</v>
       </c>
       <c r="H11" s="15" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="I11" s="16"/>
       <c r="J11" s="15">
         <v>1</v>
       </c>
       <c r="K11" s="26" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="L11" s="15"/>
     </row>
-    <row r="12" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="23">
         <f t="shared" si="0"/>
@@ -1549,10 +1548,10 @@
       </c>
       <c r="K12" s="27"/>
       <c r="L12" s="29" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="23">
         <f>ROW(B13) - ROW($B$2)</f>
@@ -1574,11 +1573,10 @@
       </c>
       <c r="K13" s="30"/>
       <c r="L13" s="29" t="s">
-        <v>155</v>
-      </c>
-      <c r="P13" s="33"/>
-    </row>
-    <row r="14" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="23">
         <f t="shared" si="0"/>
@@ -1600,7 +1598,7 @@
         <v>102</v>
       </c>
       <c r="H14" s="17" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I14" s="18"/>
       <c r="J14" s="17">
@@ -1609,7 +1607,7 @@
       <c r="K14" s="17"/>
       <c r="L14" s="17"/>
     </row>
-    <row r="15" spans="1:16" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="23">
         <f>ROW(B15) - ROW($B$2)</f>
@@ -1631,7 +1629,7 @@
         <v>81</v>
       </c>
       <c r="H15" s="15" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I15" s="16"/>
       <c r="J15" s="15">
@@ -1640,7 +1638,7 @@
       <c r="K15" s="15"/>
       <c r="L15" s="15"/>
     </row>
-    <row r="16" spans="1:16" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="23">
         <f t="shared" si="0"/>
@@ -1662,7 +1660,7 @@
         <v>103</v>
       </c>
       <c r="H16" s="17" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="I16" s="18"/>
       <c r="J16" s="17">
@@ -1693,10 +1691,10 @@
         <v>104</v>
       </c>
       <c r="H17" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I17" s="16" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="J17" s="15">
         <v>5</v>
@@ -1726,10 +1724,10 @@
         <v>105</v>
       </c>
       <c r="H18" s="17" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I18" s="18" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="J18" s="17">
         <v>1</v>
@@ -1759,10 +1757,10 @@
         <v>106</v>
       </c>
       <c r="H19" s="15" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I19" s="16" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="J19" s="15">
         <v>1</v>
@@ -1792,10 +1790,10 @@
         <v>107</v>
       </c>
       <c r="H20" s="17" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I20" s="18" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J20" s="17">
         <v>2</v>
@@ -1825,10 +1823,10 @@
         <v>108</v>
       </c>
       <c r="H21" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I21" s="16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J21" s="15">
         <v>4</v>
@@ -1858,7 +1856,7 @@
         <v>109</v>
       </c>
       <c r="H22" s="17" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="I22" s="18"/>
       <c r="J22" s="17">
@@ -1889,7 +1887,7 @@
         <v>110</v>
       </c>
       <c r="H23" s="15" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I23" s="16"/>
       <c r="J23" s="15">
@@ -1920,7 +1918,7 @@
         <v>111</v>
       </c>
       <c r="H24" s="17" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I24" s="18"/>
       <c r="J24" s="17">
@@ -1951,7 +1949,7 @@
         <v>112</v>
       </c>
       <c r="H25" s="15" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I25" s="16"/>
       <c r="J25" s="15">
@@ -1978,11 +1976,11 @@
       <c r="F26" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="G26" s="18" t="s">
-        <v>113</v>
+      <c r="G26" s="16" t="s">
+        <v>155</v>
       </c>
       <c r="H26" s="17" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="I26" s="18"/>
       <c r="J26" s="17">
@@ -2010,10 +2008,10 @@
         <v>89</v>
       </c>
       <c r="G27" s="16" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H27" s="15" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I27" s="16"/>
       <c r="J27" s="15">
@@ -2028,7 +2026,9 @@
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="C28" s="24"/>
+      <c r="C28" s="25" t="s">
+        <v>11</v>
+      </c>
       <c r="D28" s="17" t="s">
         <v>38</v>
       </c>
@@ -2042,7 +2042,7 @@
         <v>90</v>
       </c>
       <c r="H28" s="17" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="I28" s="18"/>
       <c r="J28" s="17">
@@ -2070,10 +2070,10 @@
         <v>91</v>
       </c>
       <c r="G29" s="16" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H29" s="15" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="I29" s="16"/>
       <c r="J29" s="15">
@@ -2101,10 +2101,10 @@
         <v>92</v>
       </c>
       <c r="G30" s="18" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H30" s="17" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I30" s="18"/>
       <c r="J30" s="17">
@@ -2132,10 +2132,10 @@
         <v>93</v>
       </c>
       <c r="G31" s="16" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H31" s="15" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I31" s="16"/>
       <c r="J31" s="15">
@@ -2151,27 +2151,27 @@
         <v>30</v>
       </c>
       <c r="C32" s="25" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D32" s="15"/>
       <c r="E32" s="16" t="s">
+        <v>148</v>
+      </c>
+      <c r="F32" s="15" t="s">
         <v>149</v>
       </c>
-      <c r="F32" s="15" t="s">
-        <v>150</v>
-      </c>
       <c r="G32" s="16" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H32" s="15" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="I32" s="16" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="J32" s="15"/>
       <c r="K32" s="26" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="L32" s="15"/>
     </row>
@@ -2182,27 +2182,27 @@
         <v>31</v>
       </c>
       <c r="C33" s="25" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D33" s="15"/>
       <c r="E33" s="16" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F33" s="15" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G33" s="16" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H33" s="15" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="I33" s="16" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="J33" s="15"/>
       <c r="K33" s="26" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="L33" s="15"/>
     </row>
@@ -2239,9 +2239,9 @@
     <mergeCell ref="I1:L1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="K32" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="K33" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="K11" r:id="rId3" xr:uid="{7163F1D9-70FF-4B1B-8161-0B8D0362F853}"/>
+    <hyperlink ref="K32" r:id="rId1"/>
+    <hyperlink ref="K33" r:id="rId2"/>
+    <hyperlink ref="K11" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>

</xml_diff>